<commit_message>
E9: modulo IEC 60364-5-52:2001 con tablas de fuente secundaria ABB (transcripcion cotejada), motor independiente de la norma, adaptacion del proyecto al cambiar de norma
</commit_message>
<xml_diff>
--- a/examples/reportes/memoria.xlsx
+++ b/examples/reportes/memoria.xlsx
@@ -503,7 +503,7 @@
     <t>{"text":"Potencia demandada (con el factor de demanda capturado en cada carga).","_margin":null,"_inlines":[],"_minWidth":35.87158203125,"_maxWidth":225.96875,"listMarker":{"canvas":[{"x":41.166666666666664,"y":209.06119791666666,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":204.900390625,"verticalRatio":0.3001945554748062,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Potencia demandada (con el factor de demanda capturado en cada carga).","startPosition":{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":204.900390625,"verticalRatio":0.3001945554748062,"horizontalRatio":0.010287509875351123},"pageNumbers":[4],"pages":38,"stack":false},"pageBreakCalculated":true}</t>
   </si>
   <si>
-    <t>{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común, la NOM no fija un valor).","_margin":null,"_inlines":[],"_minWidth":35.31787109375,"_maxWidth":364.71435546875,"listMarker":{"canvas":[{"x":41.166666666666664,"y":218.49479166666666,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":214.333984375,"verticalRatio":0.31847671390503873,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común, la NOM no fija un valor).","startPosition":{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":214.333984375,"verticalRatio":0.31847671390503873,"horizontalRatio":0.010287509875351123},"pageNumbers":[4],"pages":38,"stack":false},"pageBreakCalculated":true}</t>
+    <t>{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común; la norma de instalación no fija un valor).","_margin":null,"_inlines":[],"_minWidth":35.31787109375,"_maxWidth":412.8359375,"listMarker":{"canvas":[{"x":41.166666666666664,"y":218.49479166666666,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":214.333984375,"verticalRatio":0.31847671390503873,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común; la norma de instalación no fija un valor).","startPosition":{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":214.333984375,"verticalRatio":0.31847671390503873,"horizontalRatio":0.010287509875351123},"pageNumbers":[4],"pages":38,"stack":false},"pageBreakCalculated":true}</t>
   </si>
   <si>
     <t>{"text":"Transformadores, variadores y UPS se reparten equilibrados en sus tres fases de entrada.","_margin":null,"_inlines":[],"_minWidth":53.4638671875,"_maxWidth":269.650390625,"listMarker":{"canvas":[{"x":41.166666666666664,"y":227.92838541666666,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":223.767578125,"verticalRatio":0.3367588723352713,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Transformadores, variadores y UPS se reparten equilibrados en sus tres fases de entrada.","startPosition":{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":223.767578125,"verticalRatio":0.3367588723352713,"horizontalRatio":0.010287509875351123},"pageNumbers":[4],"pages":38,"stack":false},"pageBreakCalculated":true}</t>
@@ -524,7 +524,7 @@
     <t>{"text":"Potencia demandada (con el factor de demanda capturado en cada carga).","_margin":null,"_inlines":[],"_minWidth":35.87158203125,"_maxWidth":225.96875,"listMarker":{"canvas":[{"x":41.166666666666664,"y":373.0904947916667,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":368.9296875,"verticalRatio":0.6180807897286822,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Potencia demandada (con el factor de demanda capturado en cada carga).","startPosition":{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":368.9296875,"verticalRatio":0.6180807897286822,"horizontalRatio":0.010287509875351123},"pageNumbers":[4],"pages":38,"stack":false},"pageBreakCalculated":true}</t>
   </si>
   <si>
-    <t>{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común, la NOM no fija un valor).","_margin":null,"_inlines":[],"_minWidth":35.31787109375,"_maxWidth":364.71435546875,"listMarker":{"canvas":[{"x":41.166666666666664,"y":382.5240885416667,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":378.36328125,"verticalRatio":0.6363629481589147,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común, la NOM no fija un valor).","startPosition":{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":378.36328125,"verticalRatio":0.6363629481589147,"horizontalRatio":0.010287509875351123},"pageNumbers":[4],"pages":38,"stack":false},"pageBreakCalculated":true}</t>
+    <t>{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común; la norma de instalación no fija un valor).","_margin":null,"_inlines":[],"_minWidth":35.31787109375,"_maxWidth":412.8359375,"listMarker":{"canvas":[{"x":41.166666666666664,"y":382.5240885416667,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":378.36328125,"verticalRatio":0.6363629481589147,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común; la norma de instalación no fija un valor).","startPosition":{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":378.36328125,"verticalRatio":0.6363629481589147,"horizontalRatio":0.010287509875351123},"pageNumbers":[4],"pages":38,"stack":false},"pageBreakCalculated":true}</t>
   </si>
   <si>
     <t>{"text":"Transformadores, variadores y UPS se reparten equilibrados en sus tres fases de entrada.","_margin":null,"_inlines":[],"_minWidth":53.4638671875,"_maxWidth":269.650390625,"listMarker":{"canvas":[{"x":41.166666666666664,"y":391.9576822916667,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":387.796875,"verticalRatio":0.6546451065891473,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Transformadores, variadores y UPS se reparten equilibrados en sus tres fases de entrada.","startPosition":{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":387.796875,"verticalRatio":0.6546451065891473,"horizontalRatio":0.010287509875351123},"pageNumbers":[4],"pages":38,"stack":false},"pageBreakCalculated":true}</t>
@@ -542,7 +542,7 @@
     <t>{"text":"Potencia demandada (con el factor de demanda capturado en cada carga).","_margin":null,"_inlines":[],"_minWidth":35.87158203125,"_maxWidth":225.96875,"listMarker":{"canvas":[{"x":41.166666666666664,"y":522.5123697916666,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":518.3515625,"verticalRatio":0.9076580668604651,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Potencia demandada (con el factor de demanda capturado en cada carga).","startPosition":{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":518.3515625,"verticalRatio":0.9076580668604651,"horizontalRatio":0.010287509875351123},"pageNumbers":[4],"pages":38,"stack":false},"pageBreakCalculated":true}</t>
   </si>
   <si>
-    <t>{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común, la NOM no fija un valor).","_margin":null,"_inlines":[],"_minWidth":35.31787109375,"_maxWidth":364.71435546875,"listMarker":{"canvas":[{"x":41.166666666666664,"y":531.9459635416666,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":527.78515625,"verticalRatio":0.9259402252906976,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común, la NOM no fija un valor).","startPosition":{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":527.78515625,"verticalRatio":0.9259402252906976,"horizontalRatio":0.010287509875351123},"pageNumbers":[4],"pages":38,"stack":false},"pageBreakCalculated":true}</t>
+    <t>{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común; la norma de instalación no fija un valor).","_margin":null,"_inlines":[],"_minWidth":35.31787109375,"_maxWidth":412.8359375,"listMarker":{"canvas":[{"x":41.166666666666664,"y":531.9459635416666,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":527.78515625,"verticalRatio":0.9259402252906976,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común; la norma de instalación no fija un valor).","startPosition":{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":527.78515625,"verticalRatio":0.9259402252906976,"horizontalRatio":0.010287509875351123},"pageNumbers":[4],"pages":38,"stack":false},"pageBreakCalculated":true}</t>
   </si>
   <si>
     <t>TAB-A — 220 V · 3F4H</t>
@@ -554,7 +554,7 @@
     <t>{"text":"Potencia demandada (con el factor de demanda capturado en cada carga).","_margin":null,"_inlines":[],"_minWidth":35.87158203125,"_maxWidth":225.96875,"listMarker":{"canvas":[{"x":41.166666666666664,"y":171.88932291666666,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":5,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":167.728515625,"verticalRatio":0.22815603803294573,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Potencia demandada (con el factor de demanda capturado en cada carga).","startPosition":{"pageNumber":5,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":167.728515625,"verticalRatio":0.22815603803294573,"horizontalRatio":0.010287509875351123},"pageNumbers":[5],"pages":38,"stack":false},"pageBreakCalculated":true}</t>
   </si>
   <si>
-    <t>{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común, la NOM no fija un valor).","_margin":null,"_inlines":[],"_minWidth":35.31787109375,"_maxWidth":364.71435546875,"listMarker":{"canvas":[{"x":41.166666666666664,"y":181.32291666666666,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":5,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":177.162109375,"verticalRatio":0.2464381964631783,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común, la NOM no fija un valor).","startPosition":{"pageNumber":5,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":177.162109375,"verticalRatio":0.2464381964631783,"horizontalRatio":0.010287509875351123},"pageNumbers":[5],"pages":38,"stack":false},"pageBreakCalculated":true}</t>
+    <t>{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común; la norma de instalación no fija un valor).","_margin":null,"_inlines":[],"_minWidth":35.31787109375,"_maxWidth":412.8359375,"listMarker":{"canvas":[{"x":41.166666666666664,"y":181.32291666666666,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":5,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":177.162109375,"verticalRatio":0.2464381964631783,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común; la norma de instalación no fija un valor).","startPosition":{"pageNumber":5,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":177.162109375,"verticalRatio":0.2464381964631783,"horizontalRatio":0.010287509875351123},"pageNumbers":[5],"pages":38,"stack":false},"pageBreakCalculated":true}</t>
   </si>
   <si>
     <t>Elemento</t>
@@ -953,7 +953,7 @@
     <t>AL-1: Método nominal (cálculo a mano)</t>
   </si>
   <si>
-    <t>Caída de tensión (impedancia eficaz, Tabla 9 nota 2)</t>
+    <t>Caída de tensión (impedancia eficaz)</t>
   </si>
   <si>
     <t>ΔV = I · (R·cosφ + X·senφ) ;  %ΔV = ΔV / V_fn · 100</t>

</xml_diff>

<commit_message>
X/R típico (NOM-002), configuración sin calibre duplicado, tensión F-N, ayuda con imágenes y Desconectar
- Transformador: «Origen de X/R» = valor típico (pérdidas máximas NOM-002-SEDE-2010 Tabla 2,
  totales − en vacío → %R; advertencia de dato aproximado), X/R de placa o pérdidas en carga de placa.
- Cables: solo la configuración (3x#2AWG(Ph)+...), sin el renglón de calibre repetido.
- Sistemas 3F4H/1F3H: tensión L-L/L-N (220/127 V) en el inspector, el diagrama, la memoria y Excel.
- Combos con botón «?»: opciones ilustradas con fotos de Wikimedia Commons (licencia libre, con
  crédito; docs/creditos-imagenes.md) o esquemas propios; clic para elegir.
- Botón «Desconectar»: quita las conexiones de un elemento sin eliminarlo.
</commit_message>
<xml_diff>
--- a/examples/reportes/memoria.xlsx
+++ b/examples/reportes/memoria.xlsx
@@ -521,7 +521,7 @@
     <t>CG-01</t>
   </si>
   <si>
-    <t>TG — 480 V · 3F4H</t>
+    <t>TG — 480/277 V · 3F4H</t>
   </si>
   <si>
     <t>Alimenta a</t>
@@ -581,7 +581,7 @@
     <t>{"text":"Transformadores, variadores y UPS se reparten equilibrados en sus tres fases de entrada.","_margin":null,"_inlines":[],"_minWidth":53.4638671875,"_maxWidth":269.650390625,"listMarker":{"canvas":[{"x":41.166666666666664,"y":268.3580729166667,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":264.197265625,"verticalRatio":0.41511097989341084,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Transformadores, variadores y UPS se reparten equilibrados en sus tres fases de entrada.","startPosition":{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":264.197265625,"verticalRatio":0.41511097989341084,"horizontalRatio":0.010287509875351123},"pageNumbers":[4],"pages":39,"stack":false},"pageBreakCalculated":true}</t>
   </si>
   <si>
-    <t>CCM-1 — 480 V · 3F4H</t>
+    <t>CCM-1 — 480/277 V · 3F4H</t>
   </si>
   <si>
     <t>{"text":"Potencia demandada (con el factor de demanda capturado en cada carga).","_margin":null,"_inlines":[],"_minWidth":35.87158203125,"_maxWidth":225.96875,"listMarker":{"canvas":[{"x":41.166666666666664,"y":443.8424479166667,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":439.681640625,"verticalRatio":0.7551969779554264,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Potencia demandada (con el factor de demanda capturado en cada carga).","startPosition":{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":439.681640625,"verticalRatio":0.7551969779554264,"horizontalRatio":0.010287509875351123},"pageNumbers":[4],"pages":39,"stack":false},"pageBreakCalculated":true}</t>
@@ -593,7 +593,7 @@
     <t>{"text":"Transformadores, variadores y UPS se reparten equilibrados en sus tres fases de entrada.","_margin":null,"_inlines":[],"_minWidth":53.4638671875,"_maxWidth":269.650390625,"listMarker":{"canvas":[{"x":41.166666666666664,"y":462.7096354166667,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":458.548828125,"verticalRatio":0.7917612948158915,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Transformadores, variadores y UPS se reparten equilibrados en sus tres fases de entrada.","startPosition":{"pageNumber":4,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":458.548828125,"verticalRatio":0.7917612948158915,"horizontalRatio":0.010287509875351123},"pageNumbers":[4],"pages":39,"stack":false},"pageBreakCalculated":true}</t>
   </si>
   <si>
-    <t>TAB-B — 480 V · 3F4H</t>
+    <t>TAB-B — 480/277 V · 3F4H</t>
   </si>
   <si>
     <t>A</t>
@@ -605,7 +605,7 @@
     <t>{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común; la norma de instalación no fija un valor).","_margin":null,"_inlines":[],"_minWidth":35.31787109375,"_maxWidth":412.8359375,"listMarker":{"canvas":[{"x":41.166666666666664,"y":145.73893229166666,"r1":1.1666666666666667,"r2":1.1666666666666667,"type":"ellipse","color":"#666"}],"_maxWidth":7.32470703125,"_minWidth":7.32470703125,"_maxHeight":9.43359375,"_minHeight":9.43359375},"positions":[{"pageNumber":5,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":141.578125,"verticalRatio":0.17747698643410853,"horizontalRatio":0.010287509875351123}],"__height":9.43359375,"nodeInfo":{"text":"Desbalance = (F_máx − F_mín) / F_máx · 100; límite del proyecto 5 % (criterio de práctica común; la norma de instalación no fija un valor).","startPosition":{"pageNumber":5,"pageOrientation":"landscape","pageInnerHeight":516,"pageInnerWidth":712,"left":47.32470703125,"top":141.578125,"verticalRatio":0.17747698643410853,"horizontalRatio":0.010287509875351123},"pageNumbers":[5],"pages":39,"stack":false},"pageBreakCalculated":true}</t>
   </si>
   <si>
-    <t>TAB-A — 220 V · 3F4H</t>
+    <t>TAB-A — 220/127 V · 3F4H</t>
   </si>
   <si>
     <t>B</t>

</xml_diff>